<commit_message>
Updated all bom links to eu/italian resellsers
</commit_message>
<xml_diff>
--- a/hardware/bom/master_bom.xlsx
+++ b/hardware/bom/master_bom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/POLI/Magistrale/21_ACAV/F1tenth_PoliMI/hardware/bom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E5D092-A3A5-0D42-B3FE-32228A3DBCD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01780B49-EB64-6C40-A11A-738064B3CA79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="660" windowWidth="30200" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="100" yWindow="660" windowWidth="17300" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="(POLIMI) Rally + Orin Nano v1" sheetId="9" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="180">
   <si>
     <t>Scroll right to see links</t>
   </si>
@@ -641,9 +641,6 @@
     <t>Choose ONE of the listed options</t>
   </si>
   <si>
-    <t>TOTAL in the Kit = 720 pcs</t>
-  </si>
-  <si>
     <t>TOTAL in the Kit = 720 pcs (Note: ~8$ + 12$ shipping, same supplier as above so ordering together may cut costs)</t>
   </si>
   <si>
@@ -717,12 +714,6 @@
     <t>https://amzn.eu/d/04ogTQuG</t>
   </si>
   <si>
-    <t>https://a.co/d/0dyM1Yp7</t>
-  </si>
-  <si>
-    <t>https://a.co/d/01DhHfBo</t>
-  </si>
-  <si>
     <t>https://amzn.eu/d/0934urF9</t>
   </si>
   <si>
@@ -744,19 +735,10 @@
     <t>https://orders.ambimat.com/product/roboracer-power-board-multi-qty-rohs-compliant/</t>
   </si>
   <si>
-    <t>https://a.co/d/0aQPatBC</t>
-  </si>
-  <si>
-    <t>https://a.co/d/0bI2TfQP</t>
-  </si>
-  <si>
     <t>https://amzn.eu/d/04H49Gdl</t>
   </si>
   <si>
     <t>https://amzn.eu/d/0ibdH4zI</t>
-  </si>
-  <si>
-    <t>https://a.co/d/0hFfle4p</t>
   </si>
   <si>
     <t>https://amzn.eu/d/0ak3Mr9H</t>
@@ -859,7 +841,22 @@
     <t>Updated: 2026-09-24</t>
   </si>
   <si>
-    <t>s</t>
+    <t>https://amzn.eu/d/096jB5FS</t>
+  </si>
+  <si>
+    <t>https://amzn.eu/d/0dPEUR2n</t>
+  </si>
+  <si>
+    <t>https://amzn.eu/d/02tJmKlW</t>
+  </si>
+  <si>
+    <t>https://amzn.eu/d/09jG02MS</t>
+  </si>
+  <si>
+    <t>TOTAL in the Kit = 480 pcs</t>
+  </si>
+  <si>
+    <t>https://amzn.eu/d/0hnQ0stW</t>
   </si>
 </sst>
 </file>
@@ -1636,7 +1633,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="175">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1932,9 +1929,6 @@
     <xf numFmtId="0" fontId="47" fillId="5" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="6" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2019,6 +2013,36 @@
     <xf numFmtId="0" fontId="56" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2060,36 +2084,6 @@
     </xf>
     <xf numFmtId="0" fontId="46" fillId="5" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2336,25 +2330,25 @@
   <sheetData>
     <row r="1" spans="2:14" ht="17" thickBot="1"/>
     <row r="2" spans="2:14" s="95" customFormat="1" ht="23" thickBot="1">
-      <c r="B2" s="140" t="s">
+      <c r="B2" s="139" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="141" t="s">
+      <c r="C2" s="140" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="142" t="s">
-        <v>178</v>
-      </c>
-      <c r="E2" s="142" t="s">
+      <c r="D2" s="141" t="s">
+        <v>172</v>
+      </c>
+      <c r="E2" s="141" t="s">
         <v>131</v>
       </c>
-      <c r="F2" s="142" t="s">
-        <v>140</v>
-      </c>
-      <c r="G2" s="143" t="s">
+      <c r="F2" s="141" t="s">
+        <v>139</v>
+      </c>
+      <c r="G2" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="144" t="s">
+      <c r="H2" s="143" t="s">
         <v>130</v>
       </c>
       <c r="I2" s="104"/>
@@ -2364,15 +2358,15 @@
       <c r="M2" s="94"/>
     </row>
     <row r="3" spans="2:14" ht="17">
-      <c r="B3" s="134" t="s">
+      <c r="B3" s="133" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="135"/>
-      <c r="D3" s="136"/>
-      <c r="E3" s="136"/>
-      <c r="F3" s="137"/>
-      <c r="G3" s="138"/>
-      <c r="H3" s="139"/>
+      <c r="C3" s="134"/>
+      <c r="D3" s="135"/>
+      <c r="E3" s="135"/>
+      <c r="F3" s="136"/>
+      <c r="G3" s="137"/>
+      <c r="H3" s="138"/>
       <c r="I3" s="105"/>
       <c r="J3" s="60"/>
       <c r="K3" s="60"/>
@@ -2381,10 +2375,10 @@
       <c r="N3" s="61"/>
     </row>
     <row r="4" spans="2:14" ht="17">
-      <c r="B4" s="162" t="s">
-        <v>149</v>
-      </c>
-      <c r="C4" s="126">
+      <c r="B4" s="145" t="s">
+        <v>148</v>
+      </c>
+      <c r="C4" s="125">
         <v>1</v>
       </c>
       <c r="D4" s="69">
@@ -2395,11 +2389,11 @@
         <v>479.9</v>
       </c>
       <c r="F4" s="69"/>
-      <c r="G4" s="164" t="s">
-        <v>176</v>
+      <c r="G4" s="147" t="s">
+        <v>170</v>
       </c>
       <c r="H4" s="112" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="I4" s="105"/>
       <c r="J4" s="60"/>
@@ -2409,8 +2403,8 @@
       <c r="N4" s="61"/>
     </row>
     <row r="5" spans="2:14" ht="17">
-      <c r="B5" s="163"/>
-      <c r="C5" s="126">
+      <c r="B5" s="146"/>
+      <c r="C5" s="125">
         <v>1</v>
       </c>
       <c r="D5" s="69">
@@ -2421,11 +2415,11 @@
         <v>425</v>
       </c>
       <c r="F5" s="69" t="s">
-        <v>141</v>
-      </c>
-      <c r="G5" s="165"/>
+        <v>140</v>
+      </c>
+      <c r="G5" s="148"/>
       <c r="H5" s="112" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="I5" s="105"/>
       <c r="J5" s="60"/>
@@ -2435,8 +2429,8 @@
       <c r="N5" s="61"/>
     </row>
     <row r="6" spans="2:14" ht="17">
-      <c r="B6" s="163"/>
-      <c r="C6" s="126">
+      <c r="B6" s="146"/>
+      <c r="C6" s="125">
         <v>1</v>
       </c>
       <c r="D6" s="69">
@@ -2447,9 +2441,9 @@
         <v>425</v>
       </c>
       <c r="F6" s="69"/>
-      <c r="G6" s="165"/>
+      <c r="G6" s="148"/>
       <c r="H6" s="112" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="I6" s="105"/>
       <c r="J6" s="60"/>
@@ -2459,10 +2453,10 @@
       <c r="N6" s="61"/>
     </row>
     <row r="7" spans="2:14" ht="17">
-      <c r="B7" s="131" t="s">
+      <c r="B7" s="130" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="127">
+      <c r="C7" s="126">
         <v>1</v>
       </c>
       <c r="D7" s="67">
@@ -2473,11 +2467,11 @@
         <v>88.99</v>
       </c>
       <c r="F7" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G7" s="66"/>
       <c r="H7" s="113" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I7" s="106"/>
       <c r="J7" s="60"/>
@@ -2487,10 +2481,10 @@
       <c r="N7" s="61"/>
     </row>
     <row r="8" spans="2:14" ht="17">
-      <c r="B8" s="132" t="s">
+      <c r="B8" s="131" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="126">
+      <c r="C8" s="125">
         <v>1</v>
       </c>
       <c r="D8" s="69">
@@ -2501,11 +2495,11 @@
         <v>69.989999999999995</v>
       </c>
       <c r="F8" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G8" s="68"/>
       <c r="H8" s="112" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I8" s="106"/>
       <c r="J8" s="60"/>
@@ -2515,10 +2509,10 @@
       <c r="N8" s="61"/>
     </row>
     <row r="9" spans="2:14" ht="17">
-      <c r="B9" s="131" t="s">
+      <c r="B9" s="130" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="127">
+      <c r="C9" s="126">
         <v>1</v>
       </c>
       <c r="D9" s="67">
@@ -2529,7 +2523,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G9" s="66" t="s">
         <v>25</v>
@@ -2545,10 +2539,10 @@
       <c r="N9" s="61"/>
     </row>
     <row r="10" spans="2:14" ht="17">
-      <c r="B10" s="132" t="s">
+      <c r="B10" s="131" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="126">
+      <c r="C10" s="125">
         <v>1</v>
       </c>
       <c r="D10" s="69">
@@ -2559,7 +2553,7 @@
         <v>20</v>
       </c>
       <c r="F10" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G10" s="68" t="s">
         <v>32</v>
@@ -2575,10 +2569,10 @@
       <c r="N10" s="61"/>
     </row>
     <row r="11" spans="2:14" ht="17">
-      <c r="B11" s="130" t="s">
+      <c r="B11" s="129" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="125"/>
+      <c r="C11" s="124"/>
       <c r="D11" s="59"/>
       <c r="E11" s="59"/>
       <c r="F11" s="73"/>
@@ -2592,27 +2586,27 @@
       <c r="N11" s="61"/>
     </row>
     <row r="12" spans="2:14" ht="17">
-      <c r="B12" s="131" t="s">
+      <c r="B12" s="130" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="127">
+      <c r="C12" s="126">
         <v>1</v>
       </c>
       <c r="D12" s="67">
-        <v>20.32</v>
+        <v>13</v>
       </c>
       <c r="E12" s="67">
         <f t="shared" si="1"/>
-        <v>20.32</v>
+        <v>13</v>
       </c>
       <c r="F12" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G12" s="66" t="s">
-        <v>134</v>
-      </c>
-      <c r="H12" s="116" t="s">
-        <v>152</v>
+        <v>178</v>
+      </c>
+      <c r="H12" s="113" t="s">
+        <v>177</v>
       </c>
       <c r="I12" s="106"/>
       <c r="J12" s="60"/>
@@ -2622,27 +2616,27 @@
       <c r="N12" s="61"/>
     </row>
     <row r="13" spans="2:14" ht="17">
-      <c r="B13" s="132" t="s">
+      <c r="B13" s="131" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="126">
+      <c r="C13" s="125">
         <v>1</v>
       </c>
       <c r="D13" s="69">
-        <v>20.239999999999998</v>
+        <v>16</v>
       </c>
       <c r="E13" s="69">
         <f>C13*D13</f>
-        <v>20.239999999999998</v>
+        <v>16</v>
       </c>
       <c r="F13" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G13" s="68" t="s">
-        <v>135</v>
-      </c>
-      <c r="H13" s="117" t="s">
-        <v>153</v>
+        <v>134</v>
+      </c>
+      <c r="H13" s="112" t="s">
+        <v>179</v>
       </c>
       <c r="I13" s="106"/>
       <c r="J13" s="60"/>
@@ -2652,27 +2646,27 @@
       <c r="N13" s="61"/>
     </row>
     <row r="14" spans="2:14" ht="17">
-      <c r="B14" s="131" t="s">
+      <c r="B14" s="130" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="150">
+      <c r="C14" s="159">
         <v>1</v>
       </c>
-      <c r="D14" s="160">
+      <c r="D14" s="149">
         <v>12</v>
       </c>
-      <c r="E14" s="160">
+      <c r="E14" s="149">
         <f>C14*D14</f>
         <v>12</v>
       </c>
-      <c r="F14" s="160" t="s">
-        <v>141</v>
-      </c>
-      <c r="G14" s="156" t="s">
-        <v>136</v>
-      </c>
-      <c r="H14" s="158" t="s">
-        <v>154</v>
+      <c r="F14" s="149" t="s">
+        <v>140</v>
+      </c>
+      <c r="G14" s="165" t="s">
+        <v>135</v>
+      </c>
+      <c r="H14" s="167" t="s">
+        <v>151</v>
       </c>
       <c r="I14" s="106"/>
       <c r="J14" s="60"/>
@@ -2682,15 +2676,15 @@
       <c r="N14" s="61"/>
     </row>
     <row r="15" spans="2:14" ht="17">
-      <c r="B15" s="131" t="s">
+      <c r="B15" s="130" t="s">
         <v>55</v>
       </c>
-      <c r="C15" s="151"/>
-      <c r="D15" s="161"/>
-      <c r="E15" s="161"/>
-      <c r="F15" s="161"/>
-      <c r="G15" s="157"/>
-      <c r="H15" s="159"/>
+      <c r="C15" s="160"/>
+      <c r="D15" s="150"/>
+      <c r="E15" s="150"/>
+      <c r="F15" s="150"/>
+      <c r="G15" s="166"/>
+      <c r="H15" s="168"/>
       <c r="I15" s="106"/>
       <c r="J15" s="60"/>
       <c r="K15" s="60"/>
@@ -2699,27 +2693,27 @@
       <c r="N15" s="61"/>
     </row>
     <row r="16" spans="2:14" ht="17">
-      <c r="B16" s="132" t="s">
+      <c r="B16" s="131" t="s">
         <v>60</v>
       </c>
-      <c r="C16" s="126">
+      <c r="C16" s="125">
         <v>1</v>
       </c>
-      <c r="D16" s="69" t="s">
-        <v>180</v>
-      </c>
-      <c r="E16" s="69" t="e">
+      <c r="D16" s="69">
+        <v>14.39</v>
+      </c>
+      <c r="E16" s="69">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>14.39</v>
       </c>
       <c r="F16" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G16" s="68" t="s">
-        <v>137</v>
-      </c>
-      <c r="H16" s="117" t="s">
-        <v>155</v>
+        <v>136</v>
+      </c>
+      <c r="H16" s="112" t="s">
+        <v>152</v>
       </c>
       <c r="I16" s="106"/>
       <c r="J16" s="60"/>
@@ -2729,10 +2723,10 @@
       <c r="N16" s="61"/>
     </row>
     <row r="17" spans="2:29" ht="34">
-      <c r="B17" s="131" t="s">
+      <c r="B17" s="130" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="127">
+      <c r="C17" s="126">
         <v>1</v>
       </c>
       <c r="D17" s="67">
@@ -2743,13 +2737,13 @@
         <v>9.7899999999999991</v>
       </c>
       <c r="F17" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G17" s="66" t="s">
-        <v>138</v>
-      </c>
-      <c r="H17" s="116" t="s">
-        <v>156</v>
+        <v>137</v>
+      </c>
+      <c r="H17" s="113" t="s">
+        <v>153</v>
       </c>
       <c r="I17" s="106"/>
       <c r="J17" s="60"/>
@@ -2759,10 +2753,10 @@
       <c r="N17" s="61"/>
     </row>
     <row r="18" spans="2:29" ht="17">
-      <c r="B18" s="132" t="s">
+      <c r="B18" s="131" t="s">
         <v>67</v>
       </c>
-      <c r="C18" s="126">
+      <c r="C18" s="125">
         <v>1</v>
       </c>
       <c r="D18" s="69">
@@ -2773,13 +2767,13 @@
         <v>8.9</v>
       </c>
       <c r="F18" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G18" s="68" t="s">
-        <v>139</v>
-      </c>
-      <c r="H18" s="117" t="s">
-        <v>157</v>
+        <v>138</v>
+      </c>
+      <c r="H18" s="112" t="s">
+        <v>154</v>
       </c>
       <c r="I18" s="106"/>
       <c r="J18" s="60"/>
@@ -2789,15 +2783,15 @@
       <c r="N18" s="61"/>
     </row>
     <row r="19" spans="2:29" ht="17">
-      <c r="B19" s="130" t="s">
+      <c r="B19" s="129" t="s">
         <v>71</v>
       </c>
-      <c r="C19" s="128"/>
+      <c r="C19" s="127"/>
       <c r="D19" s="65"/>
       <c r="E19" s="59"/>
       <c r="F19" s="73"/>
       <c r="G19" s="64"/>
-      <c r="H19" s="118"/>
+      <c r="H19" s="117"/>
       <c r="I19" s="108"/>
       <c r="J19" s="96"/>
       <c r="K19" s="96"/>
@@ -2820,10 +2814,10 @@
       <c r="AB19" s="97"/>
     </row>
     <row r="20" spans="2:29" ht="17">
-      <c r="B20" s="131" t="s">
+      <c r="B20" s="130" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="127">
+      <c r="C20" s="126">
         <v>1</v>
       </c>
       <c r="D20" s="67">
@@ -2834,9 +2828,9 @@
         <v>355</v>
       </c>
       <c r="F20" s="67" t="s">
-        <v>141</v>
-      </c>
-      <c r="G20" s="148" t="s">
+        <v>140</v>
+      </c>
+      <c r="G20" s="157" t="s">
         <v>133</v>
       </c>
       <c r="H20" s="116" t="s">
@@ -2864,8 +2858,8 @@
       <c r="AB20" s="97"/>
     </row>
     <row r="21" spans="2:29" ht="17">
-      <c r="B21" s="131"/>
-      <c r="C21" s="127">
+      <c r="B21" s="130"/>
+      <c r="C21" s="126">
         <v>1</v>
       </c>
       <c r="D21" s="67">
@@ -2876,9 +2870,9 @@
         <v>529</v>
       </c>
       <c r="F21" s="67"/>
-      <c r="G21" s="155"/>
+      <c r="G21" s="164"/>
       <c r="H21" s="116" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I21" s="108"/>
       <c r="J21" s="96"/>
@@ -2902,10 +2896,10 @@
       <c r="AB21" s="97"/>
     </row>
     <row r="22" spans="2:29" ht="17">
-      <c r="B22" s="132" t="s">
+      <c r="B22" s="131" t="s">
         <v>77</v>
       </c>
-      <c r="C22" s="126">
+      <c r="C22" s="125">
         <v>1</v>
       </c>
       <c r="D22" s="69">
@@ -2916,11 +2910,11 @@
         <v>99</v>
       </c>
       <c r="F22" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G22" s="76"/>
-      <c r="H22" s="119" t="s">
-        <v>159</v>
+      <c r="H22" s="118" t="s">
+        <v>156</v>
       </c>
       <c r="I22" s="108"/>
       <c r="J22" s="96"/>
@@ -2945,15 +2939,15 @@
       <c r="AC22" s="97"/>
     </row>
     <row r="23" spans="2:29" ht="17">
-      <c r="B23" s="130" t="s">
-        <v>145</v>
-      </c>
-      <c r="C23" s="128"/>
+      <c r="B23" s="129" t="s">
+        <v>144</v>
+      </c>
+      <c r="C23" s="127"/>
       <c r="D23" s="65"/>
       <c r="E23" s="59"/>
       <c r="F23" s="73"/>
       <c r="G23" s="64"/>
-      <c r="H23" s="118"/>
+      <c r="H23" s="117"/>
       <c r="I23" s="108"/>
       <c r="J23" s="96"/>
       <c r="K23" s="96"/>
@@ -2977,10 +2971,10 @@
       <c r="AC23" s="97"/>
     </row>
     <row r="24" spans="2:29" ht="17">
-      <c r="B24" s="131" t="s">
+      <c r="B24" s="130" t="s">
         <v>85</v>
       </c>
-      <c r="C24" s="127">
+      <c r="C24" s="126">
         <v>1</v>
       </c>
       <c r="D24" s="67">
@@ -2991,10 +2985,10 @@
         <v>1200</v>
       </c>
       <c r="F24" s="67"/>
-      <c r="G24" s="148" t="s">
-        <v>177</v>
-      </c>
-      <c r="H24" s="120" t="s">
+      <c r="G24" s="157" t="s">
+        <v>171</v>
+      </c>
+      <c r="H24" s="119" t="s">
         <v>92</v>
       </c>
       <c r="I24" s="108"/>
@@ -3020,10 +3014,10 @@
       <c r="AC24" s="97"/>
     </row>
     <row r="25" spans="2:29" ht="17">
-      <c r="B25" s="131" t="s">
-        <v>146</v>
-      </c>
-      <c r="C25" s="127">
+      <c r="B25" s="130" t="s">
+        <v>145</v>
+      </c>
+      <c r="C25" s="126">
         <v>1</v>
       </c>
       <c r="D25" s="67">
@@ -3034,11 +3028,11 @@
         <v>535.69000000000005</v>
       </c>
       <c r="F25" s="67" t="s">
+        <v>140</v>
+      </c>
+      <c r="G25" s="158"/>
+      <c r="H25" s="116" t="s">
         <v>141</v>
-      </c>
-      <c r="G25" s="149"/>
-      <c r="H25" s="116" t="s">
-        <v>142</v>
       </c>
       <c r="I25" s="108"/>
       <c r="J25" s="96"/>
@@ -3063,10 +3057,10 @@
       <c r="AC25" s="97"/>
     </row>
     <row r="26" spans="2:29" ht="17">
-      <c r="B26" s="131" t="s">
-        <v>147</v>
-      </c>
-      <c r="C26" s="127">
+      <c r="B26" s="130" t="s">
+        <v>146</v>
+      </c>
+      <c r="C26" s="126">
         <v>1</v>
       </c>
       <c r="D26" s="67">
@@ -3077,9 +3071,9 @@
         <v>553.44000000000005</v>
       </c>
       <c r="F26" s="67"/>
-      <c r="G26" s="149"/>
+      <c r="G26" s="158"/>
       <c r="H26" s="116" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I26" s="108"/>
       <c r="J26" s="96"/>
@@ -3104,10 +3098,10 @@
       <c r="AC26" s="97"/>
     </row>
     <row r="27" spans="2:29" ht="17">
-      <c r="B27" s="131" t="s">
-        <v>148</v>
-      </c>
-      <c r="C27" s="127">
+      <c r="B27" s="130" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27" s="126">
         <v>1</v>
       </c>
       <c r="D27" s="67">
@@ -3118,9 +3112,9 @@
         <v>442.53</v>
       </c>
       <c r="F27" s="67"/>
-      <c r="G27" s="149"/>
+      <c r="G27" s="158"/>
       <c r="H27" s="116" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I27" s="108"/>
       <c r="J27" s="96"/>
@@ -3145,15 +3139,15 @@
       <c r="AC27" s="97"/>
     </row>
     <row r="28" spans="2:29" ht="17">
-      <c r="B28" s="130" t="s">
+      <c r="B28" s="129" t="s">
         <v>93</v>
       </c>
-      <c r="C28" s="128"/>
+      <c r="C28" s="127"/>
       <c r="D28" s="65"/>
       <c r="E28" s="59"/>
       <c r="F28" s="73"/>
       <c r="G28" s="64"/>
-      <c r="H28" s="118"/>
+      <c r="H28" s="117"/>
       <c r="I28" s="108"/>
       <c r="J28" s="96"/>
       <c r="K28" s="96"/>
@@ -3177,10 +3171,10 @@
       <c r="AC28" s="97"/>
     </row>
     <row r="29" spans="2:29" ht="17">
-      <c r="B29" s="132" t="s">
+      <c r="B29" s="131" t="s">
         <v>94</v>
       </c>
-      <c r="C29" s="126">
+      <c r="C29" s="125">
         <v>1</v>
       </c>
       <c r="D29" s="69">
@@ -3191,11 +3185,11 @@
         <v>110</v>
       </c>
       <c r="F29" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G29" s="77"/>
       <c r="H29" s="112" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I29" s="109"/>
       <c r="J29" s="98"/>
@@ -3220,10 +3214,10 @@
       <c r="AC29" s="97"/>
     </row>
     <row r="30" spans="2:29" ht="34">
-      <c r="B30" s="131" t="s">
+      <c r="B30" s="130" t="s">
         <v>96</v>
       </c>
-      <c r="C30" s="127">
+      <c r="C30" s="126">
         <v>1</v>
       </c>
       <c r="D30" s="67">
@@ -3234,17 +3228,17 @@
         <v>219</v>
       </c>
       <c r="F30" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G30" s="75"/>
       <c r="H30" s="113" t="s">
         <v>97</v>
       </c>
-      <c r="I30" s="152"/>
-      <c r="J30" s="152"/>
-      <c r="K30" s="152"/>
-      <c r="L30" s="152"/>
-      <c r="M30" s="153"/>
+      <c r="I30" s="161"/>
+      <c r="J30" s="161"/>
+      <c r="K30" s="161"/>
+      <c r="L30" s="161"/>
+      <c r="M30" s="162"/>
       <c r="N30" s="97"/>
       <c r="O30" s="97"/>
       <c r="P30" s="97"/>
@@ -3263,25 +3257,25 @@
       <c r="AC30" s="97"/>
     </row>
     <row r="31" spans="2:29" ht="17">
-      <c r="B31" s="132" t="s">
+      <c r="B31" s="131" t="s">
         <v>98</v>
       </c>
-      <c r="C31" s="126">
+      <c r="C31" s="125">
         <v>1</v>
       </c>
       <c r="D31" s="69">
-        <v>26.29</v>
+        <v>36.61</v>
       </c>
       <c r="E31" s="69">
         <f t="shared" si="1"/>
-        <v>26.29</v>
+        <v>36.61</v>
       </c>
       <c r="F31" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G31" s="82"/>
       <c r="H31" s="112" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="I31" s="108"/>
       <c r="J31" s="96"/>
@@ -3306,29 +3300,29 @@
       <c r="AC31" s="97"/>
     </row>
     <row r="32" spans="2:29" ht="34">
-      <c r="B32" s="131" t="s">
+      <c r="B32" s="130" t="s">
         <v>101</v>
       </c>
-      <c r="C32" s="127">
+      <c r="C32" s="126">
         <v>1</v>
       </c>
       <c r="D32" s="67">
-        <v>5.99</v>
+        <v>8.99</v>
       </c>
       <c r="E32" s="67">
         <f t="shared" si="1"/>
-        <v>5.99</v>
+        <v>8.99</v>
       </c>
       <c r="F32" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G32" s="83"/>
       <c r="H32" s="113" t="s">
-        <v>162</v>
-      </c>
-      <c r="I32" s="154"/>
-      <c r="J32" s="147"/>
-      <c r="K32" s="147"/>
+        <v>175</v>
+      </c>
+      <c r="I32" s="163"/>
+      <c r="J32" s="156"/>
+      <c r="K32" s="156"/>
       <c r="L32" s="96"/>
       <c r="M32" s="96"/>
       <c r="N32" s="97"/>
@@ -3349,10 +3343,10 @@
       <c r="AC32" s="97"/>
     </row>
     <row r="33" spans="2:29" ht="17">
-      <c r="B33" s="132" t="s">
+      <c r="B33" s="131" t="s">
         <v>103</v>
       </c>
-      <c r="C33" s="126">
+      <c r="C33" s="125">
         <v>1</v>
       </c>
       <c r="D33" s="69">
@@ -3363,13 +3357,13 @@
         <v>9.99</v>
       </c>
       <c r="F33" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G33" s="81" t="s">
         <v>104</v>
       </c>
       <c r="H33" s="112" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="I33" s="110"/>
       <c r="J33" s="99"/>
@@ -3394,10 +3388,10 @@
       <c r="AC33" s="97"/>
     </row>
     <row r="34" spans="2:29" ht="17">
-      <c r="B34" s="131" t="s">
+      <c r="B34" s="130" t="s">
         <v>106</v>
       </c>
-      <c r="C34" s="127">
+      <c r="C34" s="126">
         <v>1</v>
       </c>
       <c r="D34" s="67">
@@ -3408,13 +3402,13 @@
         <v>8.99</v>
       </c>
       <c r="F34" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G34" s="84" t="s">
         <v>104</v>
       </c>
       <c r="H34" s="113" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="I34" s="110"/>
       <c r="J34" s="99"/>
@@ -3439,25 +3433,25 @@
       <c r="AC34" s="97"/>
     </row>
     <row r="35" spans="2:29" ht="17">
-      <c r="B35" s="166" t="s">
+      <c r="B35" s="151" t="s">
         <v>108</v>
       </c>
-      <c r="C35" s="126">
+      <c r="C35" s="125">
         <v>1</v>
       </c>
       <c r="D35" s="69">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E35" s="69">
         <f t="shared" si="1"/>
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F35" s="69"/>
-      <c r="G35" s="168" t="s">
-        <v>175</v>
+      <c r="G35" s="153" t="s">
+        <v>169</v>
       </c>
       <c r="H35" s="112" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="I35" s="110"/>
       <c r="J35" s="99"/>
@@ -3482,8 +3476,8 @@
       <c r="AC35" s="97"/>
     </row>
     <row r="36" spans="2:29" ht="17">
-      <c r="B36" s="167"/>
-      <c r="C36" s="126">
+      <c r="B36" s="152"/>
+      <c r="C36" s="125">
         <v>1</v>
       </c>
       <c r="D36" s="69">
@@ -3494,11 +3488,11 @@
         <v>15.65</v>
       </c>
       <c r="F36" s="69" t="s">
-        <v>141</v>
-      </c>
-      <c r="G36" s="169"/>
+        <v>140</v>
+      </c>
+      <c r="G36" s="154"/>
       <c r="H36" s="112" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="I36" s="110"/>
       <c r="J36" s="99"/>
@@ -3523,10 +3517,10 @@
       <c r="AC36" s="97"/>
     </row>
     <row r="37" spans="2:29" ht="17">
-      <c r="B37" s="131" t="s">
+      <c r="B37" s="130" t="s">
         <v>110</v>
       </c>
-      <c r="C37" s="127">
+      <c r="C37" s="126">
         <v>1</v>
       </c>
       <c r="D37" s="67">
@@ -3537,11 +3531,11 @@
         <v>405</v>
       </c>
       <c r="F37" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G37" s="75"/>
       <c r="H37" s="113" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="I37" s="108"/>
       <c r="J37" s="96"/>
@@ -3566,15 +3560,15 @@
       <c r="AC37" s="97"/>
     </row>
     <row r="38" spans="2:29" ht="17">
-      <c r="B38" s="130" t="s">
+      <c r="B38" s="129" t="s">
         <v>112</v>
       </c>
-      <c r="C38" s="128"/>
+      <c r="C38" s="127"/>
       <c r="D38" s="65"/>
       <c r="E38" s="59"/>
       <c r="F38" s="73"/>
       <c r="G38" s="64"/>
-      <c r="H38" s="118"/>
+      <c r="H38" s="117"/>
       <c r="I38" s="108"/>
       <c r="J38" s="96"/>
       <c r="K38" s="96"/>
@@ -3598,10 +3592,10 @@
       <c r="AC38" s="97"/>
     </row>
     <row r="39" spans="2:29" ht="17">
-      <c r="B39" s="132" t="s">
+      <c r="B39" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="C39" s="126">
+      <c r="C39" s="125">
         <v>1</v>
       </c>
       <c r="D39" s="69">
@@ -3612,13 +3606,13 @@
         <v>17.43</v>
       </c>
       <c r="F39" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G39" s="68" t="s">
         <v>114</v>
       </c>
       <c r="H39" s="112" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="I39" s="108"/>
       <c r="J39" s="96"/>
@@ -3643,10 +3637,10 @@
       <c r="AC39" s="97"/>
     </row>
     <row r="40" spans="2:29" ht="17">
-      <c r="B40" s="131" t="s">
+      <c r="B40" s="130" t="s">
         <v>116</v>
       </c>
-      <c r="C40" s="127">
+      <c r="C40" s="126">
         <v>1</v>
       </c>
       <c r="D40" s="67">
@@ -3657,10 +3651,10 @@
         <v>3.38</v>
       </c>
       <c r="F40" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G40" s="85"/>
-      <c r="H40" s="120" t="s">
+      <c r="H40" s="119" t="s">
         <v>118</v>
       </c>
       <c r="I40" s="108"/>
@@ -3686,10 +3680,10 @@
       <c r="AC40" s="97"/>
     </row>
     <row r="41" spans="2:29" ht="17">
-      <c r="B41" s="132" t="s">
+      <c r="B41" s="131" t="s">
         <v>119</v>
       </c>
-      <c r="C41" s="126">
+      <c r="C41" s="125">
         <v>1</v>
       </c>
       <c r="D41" s="69">
@@ -3700,15 +3694,15 @@
         <v>10.39</v>
       </c>
       <c r="F41" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G41" s="77"/>
       <c r="H41" s="112" t="s">
-        <v>169</v>
-      </c>
-      <c r="I41" s="154"/>
-      <c r="J41" s="147"/>
-      <c r="K41" s="147"/>
+        <v>163</v>
+      </c>
+      <c r="I41" s="163"/>
+      <c r="J41" s="156"/>
+      <c r="K41" s="156"/>
       <c r="L41" s="96"/>
       <c r="M41" s="96"/>
       <c r="N41" s="97"/>
@@ -3729,10 +3723,10 @@
       <c r="AC41" s="97"/>
     </row>
     <row r="42" spans="2:29" ht="17">
-      <c r="B42" s="131" t="s">
+      <c r="B42" s="130" t="s">
         <v>121</v>
       </c>
-      <c r="C42" s="127">
+      <c r="C42" s="126">
         <v>1</v>
       </c>
       <c r="D42" s="67">
@@ -3743,17 +3737,17 @@
         <v>7.59</v>
       </c>
       <c r="F42" s="67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G42" s="66"/>
       <c r="H42" s="113" t="s">
-        <v>170</v>
-      </c>
-      <c r="I42" s="154"/>
-      <c r="J42" s="147"/>
-      <c r="K42" s="147"/>
-      <c r="L42" s="147"/>
-      <c r="M42" s="147"/>
+        <v>164</v>
+      </c>
+      <c r="I42" s="163"/>
+      <c r="J42" s="156"/>
+      <c r="K42" s="156"/>
+      <c r="L42" s="156"/>
+      <c r="M42" s="156"/>
       <c r="N42" s="97"/>
       <c r="O42" s="97"/>
       <c r="P42" s="97"/>
@@ -3772,10 +3766,10 @@
       <c r="AC42" s="97"/>
     </row>
     <row r="43" spans="2:29" ht="17">
-      <c r="B43" s="132" t="s">
+      <c r="B43" s="131" t="s">
         <v>124</v>
       </c>
-      <c r="C43" s="126">
+      <c r="C43" s="125">
         <v>1</v>
       </c>
       <c r="D43" s="69">
@@ -3786,14 +3780,14 @@
         <v>13.99</v>
       </c>
       <c r="F43" s="69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G43" s="77"/>
       <c r="H43" s="112" t="s">
-        <v>171</v>
-      </c>
-      <c r="I43" s="146"/>
-      <c r="J43" s="147"/>
+        <v>165</v>
+      </c>
+      <c r="I43" s="155"/>
+      <c r="J43" s="156"/>
       <c r="K43" s="96"/>
       <c r="L43" s="96"/>
       <c r="M43" s="96"/>
@@ -3815,20 +3809,20 @@
       <c r="AC43" s="97"/>
     </row>
     <row r="44" spans="2:29" ht="18" thickBot="1">
-      <c r="B44" s="133"/>
-      <c r="C44" s="129" t="s">
+      <c r="B44" s="132"/>
+      <c r="C44" s="128" t="s">
         <v>127</v>
       </c>
-      <c r="D44" s="121"/>
-      <c r="E44" s="121" t="e">
+      <c r="D44" s="120"/>
+      <c r="E44" s="120">
         <f>SUMIF(F4:F43, "x", E4:E43)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F44" s="122"/>
-      <c r="G44" s="123" t="s">
+        <v>2544.7599999999993</v>
+      </c>
+      <c r="F44" s="121"/>
+      <c r="G44" s="122" t="s">
         <v>128</v>
       </c>
-      <c r="H44" s="124"/>
+      <c r="H44" s="123"/>
       <c r="I44" s="106"/>
       <c r="J44" s="60"/>
       <c r="K44" s="60"/>
@@ -3852,8 +3846,8 @@
       <c r="N45" s="61"/>
     </row>
     <row r="46" spans="2:29" ht="17">
-      <c r="B46" s="145" t="s">
-        <v>179</v>
+      <c r="B46" s="144" t="s">
+        <v>173</v>
       </c>
       <c r="C46" s="62"/>
       <c r="D46" s="63"/>
@@ -6334,11 +6328,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="G4:G6"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="G35:G36"/>
     <mergeCell ref="I43:J43"/>
     <mergeCell ref="G24:G27"/>
     <mergeCell ref="C14:C15"/>
@@ -6351,6 +6340,11 @@
     <mergeCell ref="H14:H15"/>
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="G4:G6"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="G35:G36"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H20" r:id="rId1" xr:uid="{4F589D68-222B-4A43-B023-CE0E141D78F2}"/>
@@ -6363,22 +6357,28 @@
     <hyperlink ref="H8" r:id="rId8" xr:uid="{689DF752-7941-4144-8E85-2BC5EDE4EE9F}"/>
     <hyperlink ref="H7" r:id="rId9" xr:uid="{2934E811-74B4-4046-9874-E7173E570E08}"/>
     <hyperlink ref="H14:H15" r:id="rId10" display="https://amzn.eu/d/0934urF9" xr:uid="{8676A0BC-3CA7-5A4D-9375-C4DB3329C5CF}"/>
-    <hyperlink ref="H31" r:id="rId11" xr:uid="{F5D99B89-6CAA-7744-9475-E3D723F36977}"/>
-    <hyperlink ref="H32" r:id="rId12" xr:uid="{64C2AE3C-53EB-F447-A72F-B8254E0A6943}"/>
-    <hyperlink ref="H33" r:id="rId13" xr:uid="{D3DDAC29-B62D-8B48-AB0E-61B1D189861F}"/>
-    <hyperlink ref="H34" r:id="rId14" xr:uid="{2DE65291-3594-8C40-814C-4D30492506AA}"/>
-    <hyperlink ref="H36" r:id="rId15" xr:uid="{E066F5DA-2521-654D-A23E-5C0473B1DEBF}"/>
-    <hyperlink ref="H37" r:id="rId16" xr:uid="{58EBA077-E5F2-994C-8461-2CB641F3F2DD}"/>
-    <hyperlink ref="H39" r:id="rId17" xr:uid="{F414D4C9-B9F1-AB42-A1EA-7F72CE2987F0}"/>
-    <hyperlink ref="H40" r:id="rId18" xr:uid="{408FDA23-B771-5D46-B410-D154953720BF}"/>
-    <hyperlink ref="H41" r:id="rId19" xr:uid="{9F446349-F706-4F48-A3F0-4AE8C344ED77}"/>
-    <hyperlink ref="H42" r:id="rId20" xr:uid="{931E712D-264A-254F-ACE0-A9FEC29370E1}"/>
-    <hyperlink ref="H43" r:id="rId21" xr:uid="{0B1E7D38-FD1B-B84C-973D-74B46D3BD0BE}"/>
-    <hyperlink ref="H30" r:id="rId22" xr:uid="{5E2B787A-0D4D-C045-BC84-CEEBEC939FCE}"/>
-    <hyperlink ref="H29" r:id="rId23" xr:uid="{F77BF5C0-0154-FC41-9146-71EC5D057BEC}"/>
-    <hyperlink ref="H4" r:id="rId24" xr:uid="{62579853-ACC6-3F45-AB43-AB666B0CE4A5}"/>
-    <hyperlink ref="H5" r:id="rId25" xr:uid="{76B7116F-5CED-BE43-923A-75F6BB4F5B73}"/>
-    <hyperlink ref="H6" r:id="rId26" xr:uid="{270E0A71-47D3-A04D-8714-FBF827AA7557}"/>
+    <hyperlink ref="H33" r:id="rId11" xr:uid="{D3DDAC29-B62D-8B48-AB0E-61B1D189861F}"/>
+    <hyperlink ref="H34" r:id="rId12" xr:uid="{2DE65291-3594-8C40-814C-4D30492506AA}"/>
+    <hyperlink ref="H36" r:id="rId13" xr:uid="{E066F5DA-2521-654D-A23E-5C0473B1DEBF}"/>
+    <hyperlink ref="H37" r:id="rId14" xr:uid="{58EBA077-E5F2-994C-8461-2CB641F3F2DD}"/>
+    <hyperlink ref="H39" r:id="rId15" xr:uid="{F414D4C9-B9F1-AB42-A1EA-7F72CE2987F0}"/>
+    <hyperlink ref="H40" r:id="rId16" xr:uid="{408FDA23-B771-5D46-B410-D154953720BF}"/>
+    <hyperlink ref="H41" r:id="rId17" xr:uid="{9F446349-F706-4F48-A3F0-4AE8C344ED77}"/>
+    <hyperlink ref="H42" r:id="rId18" xr:uid="{931E712D-264A-254F-ACE0-A9FEC29370E1}"/>
+    <hyperlink ref="H43" r:id="rId19" xr:uid="{0B1E7D38-FD1B-B84C-973D-74B46D3BD0BE}"/>
+    <hyperlink ref="H30" r:id="rId20" xr:uid="{5E2B787A-0D4D-C045-BC84-CEEBEC939FCE}"/>
+    <hyperlink ref="H29" r:id="rId21" xr:uid="{F77BF5C0-0154-FC41-9146-71EC5D057BEC}"/>
+    <hyperlink ref="H4" r:id="rId22" xr:uid="{62579853-ACC6-3F45-AB43-AB666B0CE4A5}"/>
+    <hyperlink ref="H5" r:id="rId23" xr:uid="{76B7116F-5CED-BE43-923A-75F6BB4F5B73}"/>
+    <hyperlink ref="H6" r:id="rId24" xr:uid="{270E0A71-47D3-A04D-8714-FBF827AA7557}"/>
+    <hyperlink ref="H16" r:id="rId25" xr:uid="{971DF0EC-EE8D-0C47-81D5-EF37815C0D19}"/>
+    <hyperlink ref="H17" r:id="rId26" xr:uid="{9BCE5E90-2283-1346-9910-C49BA27E9B1E}"/>
+    <hyperlink ref="H18" r:id="rId27" xr:uid="{53E460B5-A4B1-8246-ACC0-E0B4F59AB955}"/>
+    <hyperlink ref="H31" r:id="rId28" xr:uid="{C4091FB8-58CC-8C4E-A974-5E3E367873CA}"/>
+    <hyperlink ref="H32" r:id="rId29" xr:uid="{5E006F4D-3F8F-624E-8244-07949F264730}"/>
+    <hyperlink ref="H35" r:id="rId30" xr:uid="{D6C5B699-3F20-B44E-BECC-D137DF3D9A84}"/>
+    <hyperlink ref="H12" r:id="rId31" xr:uid="{518C1E8F-4B66-D443-900D-95BD554E0194}"/>
+    <hyperlink ref="H13" r:id="rId32" xr:uid="{0EC365AA-565B-7140-9816-E9EA47F836DA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6960,14 +6960,14 @@
         <v>249.75</v>
       </c>
       <c r="D23" s="29"/>
-      <c r="E23" s="170" t="s">
+      <c r="E23" s="169" t="s">
         <v>97</v>
       </c>
-      <c r="F23" s="171"/>
-      <c r="G23" s="171"/>
-      <c r="H23" s="171"/>
-      <c r="I23" s="171"/>
-      <c r="J23" s="171"/>
+      <c r="F23" s="170"/>
+      <c r="G23" s="170"/>
+      <c r="H23" s="170"/>
+      <c r="I23" s="170"/>
+      <c r="J23" s="170"/>
       <c r="K23" s="29"/>
       <c r="L23" s="29"/>
       <c r="M23" s="29"/>
@@ -7034,12 +7034,12 @@
         <v>6.99</v>
       </c>
       <c r="D25" s="44"/>
-      <c r="E25" s="172" t="s">
+      <c r="E25" s="171" t="s">
         <v>102</v>
       </c>
-      <c r="F25" s="171"/>
-      <c r="G25" s="171"/>
-      <c r="H25" s="171"/>
+      <c r="F25" s="170"/>
+      <c r="G25" s="170"/>
+      <c r="H25" s="170"/>
       <c r="I25" s="29"/>
       <c r="J25" s="29"/>
       <c r="K25" s="29"/>
@@ -7324,12 +7324,12 @@
         <v>6.99</v>
       </c>
       <c r="D33" s="27"/>
-      <c r="E33" s="173" t="s">
+      <c r="E33" s="172" t="s">
         <v>120</v>
       </c>
-      <c r="F33" s="171"/>
-      <c r="G33" s="171"/>
-      <c r="H33" s="171"/>
+      <c r="F33" s="170"/>
+      <c r="G33" s="170"/>
+      <c r="H33" s="170"/>
       <c r="I33" s="29"/>
       <c r="J33" s="29"/>
       <c r="K33" s="29"/>
@@ -7362,14 +7362,14 @@
       <c r="D34" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="E34" s="173" t="s">
+      <c r="E34" s="172" t="s">
         <v>123</v>
       </c>
-      <c r="F34" s="171"/>
-      <c r="G34" s="171"/>
-      <c r="H34" s="171"/>
-      <c r="I34" s="171"/>
-      <c r="J34" s="171"/>
+      <c r="F34" s="170"/>
+      <c r="G34" s="170"/>
+      <c r="H34" s="170"/>
+      <c r="I34" s="170"/>
+      <c r="J34" s="170"/>
       <c r="K34" s="29"/>
       <c r="L34" s="29"/>
       <c r="M34" s="29"/>
@@ -7401,10 +7401,10 @@
       <c r="E35" s="51" t="s">
         <v>125</v>
       </c>
-      <c r="F35" s="174" t="s">
+      <c r="F35" s="173" t="s">
         <v>126</v>
       </c>
-      <c r="G35" s="171"/>
+      <c r="G35" s="170"/>
       <c r="H35" s="29"/>
       <c r="I35" s="29"/>
       <c r="J35" s="29"/>
@@ -10700,14 +10700,14 @@
         <v>0</v>
       </c>
       <c r="C6" s="7"/>
-      <c r="D6" s="175" t="s">
+      <c r="D6" s="174" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="171"/>
-      <c r="F6" s="171"/>
-      <c r="G6" s="171"/>
-      <c r="H6" s="171"/>
-      <c r="I6" s="171"/>
+      <c r="E6" s="170"/>
+      <c r="F6" s="170"/>
+      <c r="G6" s="170"/>
+      <c r="H6" s="170"/>
+      <c r="I6" s="170"/>
       <c r="J6" s="7"/>
     </row>
     <row r="7" spans="1:10" ht="15.75" customHeight="1">
@@ -10935,15 +10935,15 @@
         <v>1</v>
       </c>
       <c r="C20" s="7"/>
-      <c r="D20" s="175" t="s">
+      <c r="D20" s="174" t="s">
         <v>84</v>
       </c>
-      <c r="E20" s="171"/>
-      <c r="F20" s="171"/>
-      <c r="G20" s="171"/>
-      <c r="H20" s="171"/>
-      <c r="I20" s="171"/>
-      <c r="J20" s="171"/>
+      <c r="E20" s="170"/>
+      <c r="F20" s="170"/>
+      <c r="G20" s="170"/>
+      <c r="H20" s="170"/>
+      <c r="I20" s="170"/>
+      <c r="J20" s="170"/>
     </row>
     <row r="21" spans="1:24" ht="15.75" customHeight="1">
       <c r="A21" s="7" t="s">
@@ -10953,15 +10953,15 @@
         <v>1</v>
       </c>
       <c r="C21" s="7"/>
-      <c r="D21" s="175" t="s">
+      <c r="D21" s="174" t="s">
         <v>88</v>
       </c>
-      <c r="E21" s="171"/>
-      <c r="F21" s="171"/>
-      <c r="G21" s="171"/>
-      <c r="H21" s="171"/>
-      <c r="I21" s="171"/>
-      <c r="J21" s="171"/>
+      <c r="E21" s="170"/>
+      <c r="F21" s="170"/>
+      <c r="G21" s="170"/>
+      <c r="H21" s="170"/>
+      <c r="I21" s="170"/>
+      <c r="J21" s="170"/>
     </row>
     <row r="22" spans="1:24" ht="15.75" customHeight="1">
       <c r="A22" s="35" t="s">

</xml_diff>

<commit_message>
fix(bom): VAT-excluded total and camera spec comment
</commit_message>
<xml_diff>
--- a/hardware/bom/master_bom.xlsx
+++ b/hardware/bom/master_bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/POLI/Magistrale/21_ACAV/f1tenth_PoliMI/hardware/bom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C25656-06EC-F340-8227-D2DEED38C3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02418E1-894F-8C46-BCCD-FD479C975720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4360" yWindow="660" windowWidth="30200" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -646,51 +646,6 @@
   </si>
   <si>
     <t>https://openelab.io/products/orbbec-gemini-335l-stereo-camera?srsltid=AU7gw4WV_LMucG3H9iXtPq4gxBth5IaVVh1p7ClCoNp5OEf0dFrP1rbj</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Choose ONE of the listed cameras - </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>ONE LEFT IN STOCK</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="18"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Orbbec Gemini 335L </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>is by far the best choice. Global shutter, Stereo Vision, 60fps @ 1080p, 6DoF IMU</t>
-    </r>
   </si>
   <si>
     <t>https://www.digikey.it/it/products/detail/orbbec/100100478/23024082?srsltid=AU7gw4WokcDz96KtNyGnA0IWpYbt4VXk_WfC6iO1PVKhbTkxg6MTspV0</t>
@@ -749,6 +704,51 @@
   </si>
   <si>
     <t>Updated: 2026-10-7</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Choose ONE of the listed cameras - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ONE LEFT IN STOCK</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Orbbec Gemini 335L </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>is by far the best choice. Global shutter, Stereo Vision, 60fps @ 800p, 6DoF IMU</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2020,6 +2020,33 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2035,10 +2062,6 @@
     <xf numFmtId="0" fontId="34" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2046,32 +2069,9 @@
     <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="31" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="34" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2330,15 +2330,15 @@
   <sheetData>
     <row r="2" spans="1:8" s="74" customFormat="1" ht="47" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A2" s="95"/>
-      <c r="B2" s="178" t="s">
+      <c r="B2" s="168" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
-      <c r="H2" s="179"/>
+      <c r="C2" s="169"/>
+      <c r="D2" s="169"/>
+      <c r="E2" s="169"/>
+      <c r="F2" s="169"/>
+      <c r="G2" s="169"/>
+      <c r="H2" s="169"/>
     </row>
     <row r="3" spans="1:8" s="33" customFormat="1" ht="23" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B3" s="61" t="s">
@@ -2375,7 +2375,7 @@
       <c r="H4" s="60"/>
     </row>
     <row r="5" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B5" s="188" t="s">
+      <c r="B5" s="179" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="49">
@@ -2389,7 +2389,7 @@
         <v>479.9</v>
       </c>
       <c r="F5" s="16"/>
-      <c r="G5" s="183" t="s">
+      <c r="G5" s="175" t="s">
         <v>188</v>
       </c>
       <c r="H5" s="40" t="s">
@@ -2397,7 +2397,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B6" s="189"/>
+      <c r="B6" s="180"/>
       <c r="C6" s="49">
         <v>1</v>
       </c>
@@ -2411,13 +2411,13 @@
       <c r="F6" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="184"/>
+      <c r="G6" s="176"/>
       <c r="H6" s="40" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B7" s="189"/>
+      <c r="B7" s="180"/>
       <c r="C7" s="49">
         <v>1</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>425</v>
       </c>
       <c r="F7" s="16"/>
-      <c r="G7" s="184"/>
+      <c r="G7" s="176"/>
       <c r="H7" s="40" t="s">
         <v>13</v>
       </c>
@@ -2589,23 +2589,23 @@
       <c r="B15" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="180">
+      <c r="C15" s="170">
         <v>1</v>
       </c>
-      <c r="D15" s="173">
+      <c r="D15" s="174">
         <v>12</v>
       </c>
-      <c r="E15" s="173">
+      <c r="E15" s="174">
         <f>C15*D15</f>
         <v>12</v>
       </c>
-      <c r="F15" s="173" t="s">
+      <c r="F15" s="174" t="s">
         <v>11</v>
       </c>
-      <c r="G15" s="182" t="s">
+      <c r="G15" s="172" t="s">
         <v>32</v>
       </c>
-      <c r="H15" s="185" t="s">
+      <c r="H15" s="177" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2613,12 +2613,12 @@
       <c r="B16" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="181"/>
-      <c r="D16" s="174"/>
-      <c r="E16" s="174"/>
-      <c r="F16" s="174"/>
-      <c r="G16" s="174"/>
-      <c r="H16" s="186"/>
+      <c r="C16" s="171"/>
+      <c r="D16" s="173"/>
+      <c r="E16" s="173"/>
+      <c r="F16" s="173"/>
+      <c r="G16" s="173"/>
+      <c r="H16" s="178"/>
     </row>
     <row r="17" spans="2:17" ht="17" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B17" s="54" t="s">
@@ -2728,7 +2728,7 @@
       <c r="F21" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G21" s="177" t="s">
+      <c r="G21" s="188" t="s">
         <v>46</v>
       </c>
       <c r="H21" s="44" t="s">
@@ -2756,7 +2756,7 @@
         <v>529</v>
       </c>
       <c r="F22" s="14"/>
-      <c r="G22" s="174"/>
+      <c r="G22" s="173"/>
       <c r="H22" s="44" t="s">
         <v>48</v>
       </c>
@@ -2835,8 +2835,8 @@
         <v>1200</v>
       </c>
       <c r="F25" s="14"/>
-      <c r="G25" s="170" t="s">
-        <v>193</v>
+      <c r="G25" s="183" t="s">
+        <v>192</v>
       </c>
       <c r="H25" s="47" t="s">
         <v>53</v>
@@ -2868,7 +2868,7 @@
       <c r="F26" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G26" s="184"/>
+      <c r="G26" s="176"/>
       <c r="H26" s="44" t="s">
         <v>55</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>553.44000000000005</v>
       </c>
       <c r="F27" s="14"/>
-      <c r="G27" s="184"/>
+      <c r="G27" s="176"/>
       <c r="H27" s="44" t="s">
         <v>57</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>442.53</v>
       </c>
       <c r="F28" s="14"/>
-      <c r="G28" s="184"/>
+      <c r="G28" s="176"/>
       <c r="H28" s="44" t="s">
         <v>59</v>
       </c>
@@ -3151,7 +3151,7 @@
       <c r="Q35" s="34"/>
     </row>
     <row r="36" spans="2:17" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B36" s="175" t="s">
+      <c r="B36" s="186" t="s">
         <v>74</v>
       </c>
       <c r="C36" s="49">
@@ -3165,7 +3165,7 @@
         <v>13</v>
       </c>
       <c r="F36" s="16"/>
-      <c r="G36" s="187" t="s">
+      <c r="G36" s="189" t="s">
         <v>189</v>
       </c>
       <c r="H36" s="40" t="s">
@@ -3182,7 +3182,7 @@
       <c r="Q36" s="34"/>
     </row>
     <row r="37" spans="2:17" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B37" s="176"/>
+      <c r="B37" s="187"/>
       <c r="C37" s="49">
         <v>1</v>
       </c>
@@ -3196,7 +3196,7 @@
       <c r="F37" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="G37" s="174"/>
+      <c r="G37" s="173"/>
       <c r="H37" s="40" t="s">
         <v>76</v>
       </c>
@@ -3225,8 +3225,8 @@
         <v>405</v>
       </c>
       <c r="F38" s="14"/>
-      <c r="G38" s="170" t="s">
-        <v>191</v>
+      <c r="G38" s="183" t="s">
+        <v>196</v>
       </c>
       <c r="H38" s="41" t="s">
         <v>78</v>
@@ -3242,7 +3242,7 @@
       <c r="Q38" s="34"/>
     </row>
     <row r="39" spans="2:17" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B39" s="168" t="s">
+      <c r="B39" s="181" t="s">
         <v>79</v>
       </c>
       <c r="C39" s="50">
@@ -3258,7 +3258,7 @@
       <c r="F39" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G39" s="171"/>
+      <c r="G39" s="184"/>
       <c r="H39" s="41" t="s">
         <v>190</v>
       </c>
@@ -3273,7 +3273,7 @@
       <c r="Q39" s="34"/>
     </row>
     <row r="40" spans="2:17" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B40" s="169"/>
+      <c r="B40" s="182"/>
       <c r="C40" s="50">
         <v>1</v>
       </c>
@@ -3285,9 +3285,9 @@
         <v>408</v>
       </c>
       <c r="F40" s="14"/>
-      <c r="G40" s="172"/>
+      <c r="G40" s="185"/>
       <c r="H40" s="41" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I40" s="34"/>
       <c r="J40" s="34"/>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="F51" s="10"/>
       <c r="G51" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H51" s="164"/>
       <c r="I51" s="34"/>
@@ -3618,14 +3618,14 @@
     <row r="52" spans="2:17" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B52" s="157"/>
       <c r="C52" s="166" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D52" s="165">
         <v>0.22</v>
       </c>
       <c r="E52" s="158">
-        <f>E51*(1-D52)</f>
-        <v>2012.1971999999992</v>
+        <f>E51/(1+D52)</f>
+        <v>2114.5409836065564</v>
       </c>
       <c r="F52" s="159"/>
       <c r="G52" s="160" t="str">
@@ -3645,7 +3645,7 @@
     </row>
     <row r="54" spans="2:17" ht="17" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B54" s="66" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C54" s="9"/>
       <c r="D54" s="10"/>
@@ -5064,13 +5064,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="G5:G7"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="B5:B7"/>
     <mergeCell ref="B39:B40"/>
     <mergeCell ref="G38:G40"/>
     <mergeCell ref="F15:F16"/>
@@ -5079,6 +5072,13 @@
     <mergeCell ref="G21:G22"/>
     <mergeCell ref="G36:G37"/>
     <mergeCell ref="G25:G28"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="B5:B7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
chore(bom): fix fill colour of the camera link cell
- H39 (Gemini 335L supplier link) used a different fill from the rest of its row
</commit_message>
<xml_diff>
--- a/hardware/bom/master_bom.xlsx
+++ b/hardware/bom/master_bom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/POLI/Magistrale/21_ACAV/f1tenth_PoliMI/hardware/bom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D02418E1-894F-8C46-BCCD-FD479C975720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D641C2E-F454-0443-81A2-8850F3BD84D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="660" windowWidth="30200" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="(POLIMI) Rally + Orin Nano v1" sheetId="1" r:id="rId1"/>
@@ -1525,7 +1525,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="198">
+  <cellXfs count="199">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2093,6 +2093,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="52" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="10" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3259,7 +3262,7 @@
         <v>11</v>
       </c>
       <c r="G39" s="184"/>
-      <c r="H39" s="41" t="s">
+      <c r="H39" s="198" t="s">
         <v>190</v>
       </c>
       <c r="I39" s="34"/>

</xml_diff>